<commit_message>
Filter admin masters to used IDs
Co-authored-by: hhousni <63563021+hhousni@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/masters/master_commune.xlsx
+++ b/masters/master_commune.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$E$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$E$55</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -18,18 +19,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -43,7 +36,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -51,33 +44,15 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -440,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -451,27 +426,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>commune_name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>commune_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>prefecture_id</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>island_id</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>country_id</t>
         </is>
@@ -831,17 +806,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Cratère du Karthala</t>
+          <t>Dimani</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>KM291</t>
+          <t>KM281</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>KM29</t>
+          <t>KM28</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -858,22 +833,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Dimani</t>
+          <t>Djando</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>KM281</t>
+          <t>KM311</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>KM28</t>
+          <t>KM31</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>KM2</t>
+          <t>KM3</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -885,22 +860,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Djando</t>
+          <t>Djoumoichongo</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>KM311</t>
+          <t>KM232</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>KM31</t>
+          <t>KM23</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>KM3</t>
+          <t>KM2</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -912,17 +887,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Djoumoichongo</t>
+          <t>Djoumoipangua</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>KM232</t>
+          <t>KM221</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>KM23</t>
+          <t>KM22</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -939,17 +914,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Djoumoipangua</t>
+          <t>Domba</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>KM221</t>
+          <t>KM241</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>KM22</t>
+          <t>KM24</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -966,22 +941,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Domba</t>
+          <t>Domoni</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>KM241</t>
+          <t>KM112</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>KM24</t>
+          <t>KM11</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>KM2</t>
+          <t>KM1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -993,22 +968,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Domoni</t>
+          <t>Fomboni</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>KM112</t>
+          <t>KM321</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>KM11</t>
+          <t>KM32</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>KM1</t>
+          <t>KM3</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1020,22 +995,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Fomboni</t>
+          <t>Hamanvou</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>KM321</t>
+          <t>KM233</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>KM32</t>
+          <t>KM23</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>KM3</t>
+          <t>KM2</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1047,12 +1022,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Hamanvou</t>
+          <t>Isahari</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>KM233</t>
+          <t>KM234</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1074,17 +1049,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Isahari</t>
+          <t>Itsahidi</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>KM234</t>
+          <t>KM242</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>KM23</t>
+          <t>KM24</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1101,22 +1076,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Itsahidi</t>
+          <t>Jimlimé</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>KM242</t>
+          <t>KM113</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>KM24</t>
+          <t>KM11</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>KM2</t>
+          <t>KM1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1128,12 +1103,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Jimlimé</t>
+          <t>Koni</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>KM113</t>
+          <t>KM114</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1155,22 +1130,22 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Koni</t>
+          <t>Mbadani</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>KM114</t>
+          <t>KM235</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>KM11</t>
+          <t>KM23</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>KM1</t>
+          <t>KM2</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1182,17 +1157,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Mbadani</t>
+          <t>Mboinkou</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>KM235</t>
+          <t>KM211</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>KM23</t>
+          <t>KM21</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1209,22 +1184,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Mboinkou</t>
+          <t>Mirontsi</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>KM211</t>
+          <t>KM133</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>KM21</t>
+          <t>KM13</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>KM2</t>
+          <t>KM1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1236,22 +1211,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Mirontsi</t>
+          <t>Mitsamiouli</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>KM133</t>
+          <t>KM263</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>KM13</t>
+          <t>KM26</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>KM1</t>
+          <t>KM2</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1263,22 +1238,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Mitsamiouli</t>
+          <t>Mlédjélé</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>KM263</t>
+          <t>KM331</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>KM26</t>
+          <t>KM33</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>KM2</t>
+          <t>KM3</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1290,17 +1265,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Mlédjélé</t>
+          <t>Moili Mdjini</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>KM331</t>
+          <t>KM322</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>KM33</t>
+          <t>KM32</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1317,17 +1292,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Moili Mdjini</t>
+          <t>Moimbao</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>KM322</t>
+          <t>KM332</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>KM32</t>
+          <t>KM33</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1344,17 +1319,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Moimbao</t>
+          <t>Moimbassa</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>KM332</t>
+          <t>KM323</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>KM33</t>
+          <t>KM32</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1371,22 +1346,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Moimbassa</t>
+          <t>Moroni</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>KM323</t>
+          <t>KM274</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>KM32</t>
+          <t>KM27</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>KM3</t>
+          <t>KM2</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1398,22 +1373,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Moroni</t>
+          <t>Moya</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>KM274</t>
+          <t>KM151</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>KM27</t>
+          <t>KM15</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>KM2</t>
+          <t>KM1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1425,17 +1400,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Moya</t>
+          <t>Mramani</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>KM151</t>
+          <t>KM123</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>KM15</t>
+          <t>KM12</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1452,12 +1427,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Mramani</t>
+          <t>Mrémani</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>KM123</t>
+          <t>KM124</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1479,17 +1454,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Mrémani</t>
+          <t>Mutsamudu</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>KM124</t>
+          <t>KM134</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>KM12</t>
+          <t>KM13</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1506,17 +1481,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Mutsamudu</t>
+          <t>Ngandzalé</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>KM134</t>
+          <t>KM115</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>KM13</t>
+          <t>KM11</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1533,22 +1508,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Ngandzalé</t>
+          <t>Ngouengoe</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>KM115</t>
+          <t>KM251</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>KM11</t>
+          <t>KM25</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>KM1</t>
+          <t>KM2</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1560,12 +1535,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Ngouengoe</t>
+          <t>Nioumagama</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>KM251</t>
+          <t>KM252</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1587,17 +1562,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Nioumagama</t>
+          <t>Nyuma Komo</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>KM252</t>
+          <t>KM264</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>KM25</t>
+          <t>KM26</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1614,17 +1589,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Nyuma Komo</t>
+          <t>Nyuma Mro</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>KM264</t>
+          <t>KM212</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>KM26</t>
+          <t>KM21</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1641,12 +1616,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Nyuma Mro</t>
+          <t>Nyuma Msiru</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>KM212</t>
+          <t>KM213</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1668,17 +1643,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Nyuma Msiru</t>
+          <t>Nyumamro Kiblani</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>KM213</t>
+          <t>KM265</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>KM21</t>
+          <t>KM26</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1695,12 +1670,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Nyumamro Kiblani</t>
+          <t>Nyumamro Souheili</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>KM265</t>
+          <t>KM266</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1722,17 +1697,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Nyumamro Souheili</t>
+          <t>Oichili Yadjou</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>KM266</t>
+          <t>KM282</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>KM26</t>
+          <t>KM28</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1749,12 +1724,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Oichili Yadjou</t>
+          <t>Oichili Yamboini</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>KM282</t>
+          <t>KM283</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1776,22 +1751,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Oichili Yamboini</t>
+          <t>Ongojou</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>KM283</t>
+          <t>KM125</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>KM28</t>
+          <t>KM12</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>KM2</t>
+          <t>KM1</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -1803,17 +1778,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Ongojou</t>
+          <t>Ouani</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>KM125</t>
+          <t>KM143</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>KM12</t>
+          <t>KM14</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1830,22 +1805,22 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Ouani</t>
+          <t>Pimba</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>KM143</t>
+          <t>KM243</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>KM14</t>
+          <t>KM24</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>KM1</t>
+          <t>KM2</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -1857,22 +1832,22 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Pimba</t>
+          <t>Sima</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>KM243</t>
+          <t>KM152</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>KM24</t>
+          <t>KM15</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>KM2</t>
+          <t>KM1</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -1884,22 +1859,22 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Sima</t>
+          <t>Tsinimoipangua</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>KM152</t>
+          <t>KM222</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>KM15</t>
+          <t>KM22</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>KM1</t>
+          <t>KM2</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -1911,22 +1886,22 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Tsinimoipangua</t>
+          <t>Vouani</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>KM222</t>
+          <t>KM153</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>KM22</t>
+          <t>KM15</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>KM2</t>
+          <t>KM1</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -1935,35 +1910,8 @@
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Vouani</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>KM153</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>KM15</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>KM1</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>KM</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E56"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <autoFilter ref="A1:E55"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>